<commit_message>
Some more item domain work
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/BJ's/BJ's_Bakery_20260531.xlsx
+++ b/WorkBot/main/data/orders/BJ's/BJ's_Bakery_20260531.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,44 @@
         <v>101.97</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>88867012959</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Employee Water - Office</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6.69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Celsius - Vibe Peach, Tropical, Arctic</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="E8" t="n">
+        <v>199.43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>